<commit_message>
fix: english audio 12:00 am is played for midnight
</commit_message>
<xml_diff>
--- a/original/en/english_audio_list.xlsx
+++ b/original/en/english_audio_list.xlsx
@@ -17,15 +17,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>am</t>
   </si>
   <si>
     <t>pm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">it is midnight</t>
   </si>
   <si>
     <t xml:space="preserve">it is 1</t>
@@ -154,14 +151,11 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyProtection="1">
@@ -650,408 +644,403 @@
   </cols>
   <sheetData>
     <row r="1" ht="15">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" ht="15">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" ht="15">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" ht="15">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" ht="15">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" ht="15">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" ht="15">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" ht="15">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" ht="15">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" ht="15">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" ht="15">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" ht="15">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" ht="15">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" ht="15">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" ht="15">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" ht="15">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" ht="15">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" ht="15">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" ht="15">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" ht="15">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" ht="15">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" ht="15">
+      <c r="A25" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" ht="15">
+      <c r="A26" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" ht="15">
+      <c r="A27" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="15">
+      <c r="A28" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" ht="15">
+      <c r="A29" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" ht="15">
+      <c r="A30" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" ht="15">
+      <c r="A31" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" ht="15">
+      <c r="A32" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33" ht="15">
+      <c r="A33" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" ht="15">
+      <c r="A34" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" ht="15">
+      <c r="A35" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" ht="15">
+      <c r="A36" s="2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" ht="15">
+      <c r="A37" s="2">
         <v>23</v>
       </c>
     </row>
-    <row r="25" ht="15">
-      <c r="A25" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="26" ht="15">
-      <c r="A26" s="3">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" ht="15">
-      <c r="A27" s="3">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="28" ht="15">
-      <c r="A28" s="3">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" ht="15">
-      <c r="A29" s="3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" ht="15">
-      <c r="A30" s="3">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" ht="15">
-      <c r="A31" s="3">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" ht="15">
-      <c r="A32" s="3">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" ht="15">
-      <c r="A33" s="3">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="34" ht="15">
-      <c r="A34" s="3">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="35" ht="15">
-      <c r="A35" s="3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36" ht="15">
-      <c r="A36" s="3">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="37" ht="15">
-      <c r="A37" s="3">
-        <v>22</v>
-      </c>
-    </row>
     <row r="38" ht="15">
-      <c r="A38" s="3">
+      <c r="A38" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" ht="15">
+      <c r="A39" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" ht="15">
+      <c r="A40" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" ht="15">
+      <c r="A41" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" ht="15">
+      <c r="A42" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" ht="15">
+      <c r="A43" s="2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" ht="15">
+      <c r="A44" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" ht="15">
+      <c r="A45" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="46" ht="15">
+      <c r="A46" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" ht="15">
+      <c r="A47" s="2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="48" ht="15">
+      <c r="A48" s="2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="49" ht="15">
+      <c r="A49" s="2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" ht="15">
+      <c r="A50" s="2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="51" ht="15">
+      <c r="A51" s="2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="52" ht="15">
+      <c r="A52" s="2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" ht="15">
+      <c r="A53" s="2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="54" ht="15">
+      <c r="A54" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55" ht="15">
+      <c r="A55" s="2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" ht="15">
+      <c r="A56" s="2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="57" ht="15">
+      <c r="A57" s="2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" ht="15">
+      <c r="A58" s="2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="59" ht="15">
+      <c r="A59" s="2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="60" ht="15">
+      <c r="A60" s="2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="61" ht="15">
+      <c r="A61" s="2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="62" ht="15">
+      <c r="A62" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="63" ht="14.25">
+      <c r="A63" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="64" ht="14.25">
+      <c r="A64" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="65" ht="14.25">
+      <c r="A65" s="2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="66" ht="14.25">
+      <c r="A66" s="2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="67" ht="14.25">
+      <c r="A67" s="2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="68" ht="14.25">
+      <c r="A68" s="2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="69" ht="14.25">
+      <c r="A69" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="70" ht="14.25">
+      <c r="A70" s="2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="71" ht="14.25">
+      <c r="A71" s="2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="72" ht="14.25">
+      <c r="A72" s="2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="73" ht="14.25">
+      <c r="A73" s="2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="74" ht="14.25">
+      <c r="A74" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" ht="15">
-      <c r="A39" s="3">
+    <row r="75" ht="14.25">
+      <c r="A75" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="40" ht="15">
-      <c r="A40" s="3">
+    <row r="76" ht="14.25">
+      <c r="A76" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="41" ht="15">
-      <c r="A41" s="3">
+    <row r="77" ht="14.25">
+      <c r="A77" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="42" ht="15">
-      <c r="A42" s="3">
+    <row r="78" ht="14.25">
+      <c r="A78" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="43" ht="15">
-      <c r="A43" s="3">
+    <row r="79" ht="14.25">
+      <c r="A79" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="44" ht="15">
-      <c r="A44" s="3">
+    <row r="80" ht="14.25">
+      <c r="A80" s="2" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="45" ht="15">
-      <c r="A45" s="3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="46" ht="15">
-      <c r="A46" s="3">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="47" ht="15">
-      <c r="A47" s="3">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="48" ht="15">
-      <c r="A48" s="3">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="49" ht="15">
-      <c r="A49" s="3">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="50" ht="15">
-      <c r="A50" s="3">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="51" ht="15">
-      <c r="A51" s="3">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="52" ht="15">
-      <c r="A52" s="3">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="53" ht="15">
-      <c r="A53" s="3">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="54" ht="15">
-      <c r="A54" s="3">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="55" ht="15">
-      <c r="A55" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="56" ht="15">
-      <c r="A56" s="3">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="57" ht="15">
-      <c r="A57" s="3">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="58" ht="15">
-      <c r="A58" s="3">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="59" ht="15">
-      <c r="A59" s="3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="60" ht="15">
-      <c r="A60" s="3">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="61" ht="15">
-      <c r="A61" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="62" ht="15">
-      <c r="A62" s="3">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="63" ht="15">
-      <c r="A63" s="3">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="64" ht="14.25">
-      <c r="A64" s="3">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="65" ht="14.25">
-      <c r="A65" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="66" ht="14.25">
-      <c r="A66" s="3">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="67" ht="14.25">
-      <c r="A67" s="3">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="68" ht="14.25">
-      <c r="A68" s="3">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="69" ht="14.25">
-      <c r="A69" s="3">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="70" ht="14.25">
-      <c r="A70" s="3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="71" ht="14.25">
-      <c r="A71" s="3">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="72" ht="14.25">
-      <c r="A72" s="3">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="73" ht="14.25">
-      <c r="A73" s="3">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="74" ht="14.25">
-      <c r="A74" s="3">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="75" ht="14.25">
-      <c r="A75" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="76" ht="14.25">
-      <c r="A76" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="77" ht="14.25">
-      <c r="A77" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="78" ht="14.25">
-      <c r="A78" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="79" ht="14.25">
-      <c r="A79" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="80" ht="14.25">
-      <c r="A80" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="81" ht="14.25">
-      <c r="A81" s="3" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>